<commit_message>
[ADD] Datos adicionales, Columna en Solicitudes Calculadas
</commit_message>
<xml_diff>
--- a/Estudio.Controllers/Files/Solicitudes Calculadas.xlsx
+++ b/Estudio.Controllers/Files/Solicitudes Calculadas.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25831"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\Vida Camara\Solucion\Cotizador\EstudioVidaCamara\Estudio.Controllers\Files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\VivirSeguros\RENTA VITALICIA\vivirseguros.cotizador-rv.mvc\Estudio.Controllers\Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBAF15F2-E5D6-4AA2-B91A-0ED579199AA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="26025" windowHeight="8670"/>
+    <workbookView xWindow="21480" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Solicitudes Calculadas" sheetId="1" r:id="rId1"/>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="29">
   <si>
     <t>Cobertura</t>
   </si>
@@ -109,12 +110,15 @@
   </si>
   <si>
     <t>Descripción del Error</t>
+  </si>
+  <si>
+    <t>Departamento</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="#,##0.000000"/>
     <numFmt numFmtId="165" formatCode="#,##0.00000"/>
@@ -486,8 +490,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Y1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:Z1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.28515625" style="4" customWidth="1"/>
@@ -514,9 +518,10 @@
     <col min="23" max="23" width="18.7109375" style="17" customWidth="1"/>
     <col min="24" max="24" width="11.85546875" style="7" customWidth="1"/>
     <col min="25" max="25" width="14" style="17" customWidth="1"/>
+    <col min="26" max="26" width="15.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:26" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>15</v>
       </c>
@@ -591,6 +596,9 @@
       </c>
       <c r="Y1" s="2" t="s">
         <v>14</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -600,7 +608,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:P1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>

<commit_message>
[ADD] News columns Report Solicitudes Calculadas
</commit_message>
<xml_diff>
--- a/Estudio.Controllers/Files/Solicitudes Calculadas.xlsx
+++ b/Estudio.Controllers/Files/Solicitudes Calculadas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25831"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26501"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\VivirSeguros\RENTA VITALICIA\vivirseguros.cotizador-rv.mvc\Estudio.Controllers\Files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\VIVIR SEGUROS\vivirseguros.cotizador-rv.mvc\Estudio.Controllers\Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBAF15F2-E5D6-4AA2-B91A-0ED579199AA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F53C010F-8942-441D-96F9-D42A386C26CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="21480" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Solicitudes Calculadas" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="33">
   <si>
     <t>Cobertura</t>
   </si>
@@ -113,6 +113,18 @@
   </si>
   <si>
     <t>Departamento</t>
+  </si>
+  <si>
+    <t>Departamento Cotizador</t>
+  </si>
+  <si>
+    <t>Asesor</t>
+  </si>
+  <si>
+    <t>Supervisor</t>
+  </si>
+  <si>
+    <t>Departamento Jubilare</t>
   </si>
 </sst>
 </file>
@@ -491,7 +503,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z1"/>
+  <dimension ref="A1:AD1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.28515625" style="4" customWidth="1"/>
@@ -521,7 +533,7 @@
     <col min="26" max="26" width="15.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>15</v>
       </c>
@@ -599,6 +611,18 @@
       </c>
       <c r="Z1" s="1" t="s">
         <v>28</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AB1" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="AC1" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="AD1" s="2" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -609,7 +633,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:T1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.28515625" style="4" customWidth="1"/>
@@ -630,7 +654,7 @@
     <col min="16" max="16" width="54.7109375" style="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>16</v>
       </c>
@@ -678,6 +702,18 @@
       </c>
       <c r="P1" s="2" t="s">
         <v>27</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>